<commit_message>
Add Vercel deployment with Blob Storage, admin upload, and dashboard fixes
- Restructured project for Vercel: public/index.html, api routes, vercel.json
- Added password-protected admin upload with SVG icon states
- Blob Storage integration for persistent dashboard data
- Fixed charts breaking on new customer rows with empty cells
- Fixed Excel error values (#REF!, #N/A, etc.) treated as null
- Added filter ordering, Clear button, and raised filter cap to 50
- Updated selftest with new customer row and error handling tests
</commit_message>
<xml_diff>
--- a/Dashboard 1.xlsx
+++ b/Dashboard 1.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Nithin\Vendor tracker\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BB294924-1356-460F-BC56-8FE5C9B3FC62}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C91BBDB1-13BD-440A-BBF4-AE7BDEA3B2BC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -45,7 +45,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="58" uniqueCount="37">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="59" uniqueCount="38">
   <si>
     <t>Customer Name</t>
   </si>
@@ -156,6 +156,9 @@
   </si>
   <si>
     <t>Pending Quantity (Nos)</t>
+  </si>
+  <si>
+    <t>Clearance Given tip Stores(MW)</t>
   </si>
 </sst>
 </file>
@@ -394,13 +397,13 @@
               <c:extLst>
                 <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
                   <c15:fullRef>
-                    <c15:sqref>Sheet2!$G$3:$W$3</c15:sqref>
+                    <c15:sqref>Sheet2!$G$3:$X$3</c15:sqref>
                   </c15:fullRef>
                 </c:ext>
               </c:extLst>
-              <c:f>Sheet2!$G$3:$Q$3</c:f>
+              <c:f>(Sheet2!$G$3:$Q$3,Sheet2!$X$3)</c:f>
               <c:strCache>
-                <c:ptCount val="11"/>
+                <c:ptCount val="12"/>
                 <c:pt idx="0">
                   <c:v>PO Quantity (Nos)</c:v>
                 </c:pt>
@@ -434,6 +437,9 @@
                 <c:pt idx="10">
                   <c:v>Stock(MW)</c:v>
                 </c:pt>
+                <c:pt idx="11">
+                  <c:v>BOE Acceptance Pending </c:v>
+                </c:pt>
               </c:strCache>
             </c:strRef>
           </c:cat>
@@ -442,14 +448,14 @@
               <c:extLst>
                 <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
                   <c15:fullRef>
-                    <c15:sqref>Sheet2!$G$4:$W$4</c15:sqref>
+                    <c15:sqref>Sheet2!$G$4:$X$4</c15:sqref>
                   </c15:fullRef>
                 </c:ext>
               </c:extLst>
-              <c:f>Sheet2!$G$4:$Q$4</c:f>
+              <c:f>(Sheet2!$G$4:$Q$4,Sheet2!$X$4)</c:f>
               <c:numCache>
                 <c:formatCode>0</c:formatCode>
-                <c:ptCount val="11"/>
+                <c:ptCount val="12"/>
                 <c:pt idx="0" formatCode="General">
                   <c:v>406505</c:v>
                 </c:pt>
@@ -467,6 +473,9 @@
                 </c:pt>
                 <c:pt idx="8" formatCode="0.00">
                   <c:v>109.682175</c:v>
+                </c:pt>
+                <c:pt idx="11" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)">
+                  <c:v>1135435832.9599979</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -539,15 +548,15 @@
                     <c:extLst>
                       <c:ext uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
                         <c15:fullRef>
-                          <c15:sqref>Sheet2!$G$3:$W$3</c15:sqref>
+                          <c15:sqref>Sheet2!$G$3:$X$3</c15:sqref>
                         </c15:fullRef>
                         <c15:formulaRef>
-                          <c15:sqref>Sheet2!$G$3:$Q$3</c15:sqref>
+                          <c15:sqref>(Sheet2!$G$3:$Q$3,Sheet2!$X$3)</c15:sqref>
                         </c15:formulaRef>
                       </c:ext>
                     </c:extLst>
                     <c:strCache>
-                      <c:ptCount val="11"/>
+                      <c:ptCount val="12"/>
                       <c:pt idx="0">
                         <c:v>PO Quantity (Nos)</c:v>
                       </c:pt>
@@ -580,6 +589,9 @@
                       </c:pt>
                       <c:pt idx="10">
                         <c:v>Stock(MW)</c:v>
+                      </c:pt>
+                      <c:pt idx="11">
+                        <c:v>BOE Acceptance Pending </c:v>
                       </c:pt>
                     </c:strCache>
                   </c:strRef>
@@ -589,16 +601,16 @@
                     <c:extLst>
                       <c:ext uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
                         <c15:fullRef>
-                          <c15:sqref>Sheet2!$G$5:$W$5</c15:sqref>
+                          <c15:sqref>Sheet2!$G$5:$X$5</c15:sqref>
                         </c15:fullRef>
                         <c15:formulaRef>
-                          <c15:sqref>Sheet2!$G$5:$Q$5</c15:sqref>
+                          <c15:sqref>(Sheet2!$G$5:$Q$5,Sheet2!$X$5)</c15:sqref>
                         </c15:formulaRef>
                       </c:ext>
                     </c:extLst>
                     <c:numCache>
                       <c:formatCode>General</c:formatCode>
-                      <c:ptCount val="11"/>
+                      <c:ptCount val="12"/>
                       <c:pt idx="0">
                         <c:v>1860</c:v>
                       </c:pt>
@@ -675,15 +687,15 @@
                     <c:extLst>
                       <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
                         <c15:fullRef>
-                          <c15:sqref>Sheet2!$G$3:$W$3</c15:sqref>
+                          <c15:sqref>Sheet2!$G$3:$X$3</c15:sqref>
                         </c15:fullRef>
                         <c15:formulaRef>
-                          <c15:sqref>Sheet2!$G$3:$Q$3</c15:sqref>
+                          <c15:sqref>(Sheet2!$G$3:$Q$3,Sheet2!$X$3)</c15:sqref>
                         </c15:formulaRef>
                       </c:ext>
                     </c:extLst>
                     <c:strCache>
-                      <c:ptCount val="11"/>
+                      <c:ptCount val="12"/>
                       <c:pt idx="0">
                         <c:v>PO Quantity (Nos)</c:v>
                       </c:pt>
@@ -716,6 +728,9 @@
                       </c:pt>
                       <c:pt idx="10">
                         <c:v>Stock(MW)</c:v>
+                      </c:pt>
+                      <c:pt idx="11">
+                        <c:v>BOE Acceptance Pending </c:v>
                       </c:pt>
                     </c:strCache>
                   </c:strRef>
@@ -725,16 +740,16 @@
                     <c:extLst>
                       <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
                         <c15:fullRef>
-                          <c15:sqref>Sheet2!$G$6:$W$6</c15:sqref>
+                          <c15:sqref>Sheet2!$G$6:$X$6</c15:sqref>
                         </c15:fullRef>
                         <c15:formulaRef>
-                          <c15:sqref>Sheet2!$G$6:$Q$6</c15:sqref>
+                          <c15:sqref>(Sheet2!$G$6:$Q$6,Sheet2!$X$6)</c15:sqref>
                         </c15:formulaRef>
                       </c:ext>
                     </c:extLst>
                     <c:numCache>
                       <c:formatCode>0</c:formatCode>
-                      <c:ptCount val="11"/>
+                      <c:ptCount val="12"/>
                       <c:pt idx="0" formatCode="General">
                         <c:v>40000</c:v>
                       </c:pt>
@@ -811,15 +826,15 @@
                     <c:extLst>
                       <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
                         <c15:fullRef>
-                          <c15:sqref>Sheet2!$G$3:$W$3</c15:sqref>
+                          <c15:sqref>Sheet2!$G$3:$X$3</c15:sqref>
                         </c15:fullRef>
                         <c15:formulaRef>
-                          <c15:sqref>Sheet2!$G$3:$Q$3</c15:sqref>
+                          <c15:sqref>(Sheet2!$G$3:$Q$3,Sheet2!$X$3)</c15:sqref>
                         </c15:formulaRef>
                       </c:ext>
                     </c:extLst>
                     <c:strCache>
-                      <c:ptCount val="11"/>
+                      <c:ptCount val="12"/>
                       <c:pt idx="0">
                         <c:v>PO Quantity (Nos)</c:v>
                       </c:pt>
@@ -852,6 +867,9 @@
                       </c:pt>
                       <c:pt idx="10">
                         <c:v>Stock(MW)</c:v>
+                      </c:pt>
+                      <c:pt idx="11">
+                        <c:v>BOE Acceptance Pending </c:v>
                       </c:pt>
                     </c:strCache>
                   </c:strRef>
@@ -861,16 +879,16 @@
                     <c:extLst>
                       <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
                         <c15:fullRef>
-                          <c15:sqref>Sheet2!$G$7:$W$7</c15:sqref>
+                          <c15:sqref>Sheet2!$G$7:$X$7</c15:sqref>
                         </c15:fullRef>
                         <c15:formulaRef>
-                          <c15:sqref>Sheet2!$G$7:$Q$7</c15:sqref>
+                          <c15:sqref>(Sheet2!$G$7:$Q$7,Sheet2!$X$7)</c15:sqref>
                         </c15:formulaRef>
                       </c:ext>
                     </c:extLst>
                     <c:numCache>
                       <c:formatCode>0</c:formatCode>
-                      <c:ptCount val="11"/>
+                      <c:ptCount val="12"/>
                       <c:pt idx="0" formatCode="General">
                         <c:v>3720</c:v>
                       </c:pt>
@@ -947,15 +965,15 @@
                     <c:extLst>
                       <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
                         <c15:fullRef>
-                          <c15:sqref>Sheet2!$G$3:$W$3</c15:sqref>
+                          <c15:sqref>Sheet2!$G$3:$X$3</c15:sqref>
                         </c15:fullRef>
                         <c15:formulaRef>
-                          <c15:sqref>Sheet2!$G$3:$Q$3</c15:sqref>
+                          <c15:sqref>(Sheet2!$G$3:$Q$3,Sheet2!$X$3)</c15:sqref>
                         </c15:formulaRef>
                       </c:ext>
                     </c:extLst>
                     <c:strCache>
-                      <c:ptCount val="11"/>
+                      <c:ptCount val="12"/>
                       <c:pt idx="0">
                         <c:v>PO Quantity (Nos)</c:v>
                       </c:pt>
@@ -988,6 +1006,9 @@
                       </c:pt>
                       <c:pt idx="10">
                         <c:v>Stock(MW)</c:v>
+                      </c:pt>
+                      <c:pt idx="11">
+                        <c:v>BOE Acceptance Pending </c:v>
                       </c:pt>
                     </c:strCache>
                   </c:strRef>
@@ -997,16 +1018,16 @@
                     <c:extLst>
                       <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
                         <c15:fullRef>
-                          <c15:sqref>Sheet2!$G$8:$W$8</c15:sqref>
+                          <c15:sqref>Sheet2!$G$8:$X$8</c15:sqref>
                         </c15:fullRef>
                         <c15:formulaRef>
-                          <c15:sqref>Sheet2!$G$8:$Q$8</c15:sqref>
+                          <c15:sqref>(Sheet2!$G$8:$Q$8,Sheet2!$X$8)</c15:sqref>
                         </c15:formulaRef>
                       </c:ext>
                     </c:extLst>
                     <c:numCache>
                       <c:formatCode>General</c:formatCode>
-                      <c:ptCount val="11"/>
+                      <c:ptCount val="12"/>
                       <c:pt idx="0">
                         <c:v>144320</c:v>
                       </c:pt>
@@ -1083,15 +1104,15 @@
                     <c:extLst>
                       <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
                         <c15:fullRef>
-                          <c15:sqref>Sheet2!$G$3:$W$3</c15:sqref>
+                          <c15:sqref>Sheet2!$G$3:$X$3</c15:sqref>
                         </c15:fullRef>
                         <c15:formulaRef>
-                          <c15:sqref>Sheet2!$G$3:$Q$3</c15:sqref>
+                          <c15:sqref>(Sheet2!$G$3:$Q$3,Sheet2!$X$3)</c15:sqref>
                         </c15:formulaRef>
                       </c:ext>
                     </c:extLst>
                     <c:strCache>
-                      <c:ptCount val="11"/>
+                      <c:ptCount val="12"/>
                       <c:pt idx="0">
                         <c:v>PO Quantity (Nos)</c:v>
                       </c:pt>
@@ -1124,6 +1145,9 @@
                       </c:pt>
                       <c:pt idx="10">
                         <c:v>Stock(MW)</c:v>
+                      </c:pt>
+                      <c:pt idx="11">
+                        <c:v>BOE Acceptance Pending </c:v>
                       </c:pt>
                     </c:strCache>
                   </c:strRef>
@@ -1133,16 +1157,16 @@
                     <c:extLst>
                       <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
                         <c15:fullRef>
-                          <c15:sqref>Sheet2!$G$9:$W$9</c15:sqref>
+                          <c15:sqref>Sheet2!$G$9:$X$9</c15:sqref>
                         </c15:fullRef>
                         <c15:formulaRef>
-                          <c15:sqref>Sheet2!$G$9:$Q$9</c15:sqref>
+                          <c15:sqref>(Sheet2!$G$9:$Q$9,Sheet2!$X$9)</c15:sqref>
                         </c15:formulaRef>
                       </c:ext>
                     </c:extLst>
                     <c:numCache>
                       <c:formatCode>0</c:formatCode>
-                      <c:ptCount val="11"/>
+                      <c:ptCount val="12"/>
                       <c:pt idx="0" formatCode="General">
                         <c:v>20088</c:v>
                       </c:pt>
@@ -2502,7 +2526,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{296D20F1-4FAA-4DF4-B015-8406C76F51DD}">
-  <dimension ref="B3:W12"/>
+  <dimension ref="B3:X12"/>
   <sheetFormatPr defaultColWidth="8.90625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="8.90625" style="1"/>
@@ -2521,16 +2545,17 @@
     <col min="15" max="15" width="22" style="1" bestFit="1" customWidth="1"/>
     <col min="16" max="16" width="19" style="1" bestFit="1" customWidth="1"/>
     <col min="17" max="17" width="16.6328125" style="1" customWidth="1"/>
-    <col min="18" max="18" width="16.36328125" style="1" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="18.90625" style="1" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="18.81640625" style="1" customWidth="1"/>
-    <col min="21" max="21" width="21.08984375" style="1" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="26" style="1" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="22.453125" style="1" bestFit="1" customWidth="1"/>
-    <col min="24" max="16384" width="8.90625" style="1"/>
+    <col min="18" max="18" width="27.81640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="16.36328125" style="1" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="18.90625" style="1" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="18.81640625" style="1" customWidth="1"/>
+    <col min="22" max="22" width="21.08984375" style="1" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="26" style="1" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="22.453125" style="1" bestFit="1" customWidth="1"/>
+    <col min="25" max="16384" width="8.90625" style="1"/>
   </cols>
   <sheetData>
-    <row r="3" spans="2:23" s="4" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="3" spans="2:24" s="4" customFormat="1" x14ac:dyDescent="0.35">
       <c r="B3" s="4" t="s">
         <v>0</v>
       </c>
@@ -2580,25 +2605,28 @@
         <v>26</v>
       </c>
       <c r="R3" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="S3" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="S3" s="4" t="s">
+      <c r="T3" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="T3" s="4" t="s">
+      <c r="U3" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="U3" s="4" t="s">
+      <c r="V3" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="V3" s="4" t="s">
+      <c r="W3" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="W3" s="4" t="s">
+      <c r="X3" s="4" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="4" spans="2:23" x14ac:dyDescent="0.35">
+    <row r="4" spans="2:24" x14ac:dyDescent="0.35">
       <c r="B4" s="1" t="s">
         <v>8</v>
       </c>
@@ -2643,30 +2671,31 @@
       </c>
       <c r="P4" s="3"/>
       <c r="Q4" s="3"/>
-      <c r="R4" s="5">
+      <c r="R4" s="3"/>
+      <c r="S4" s="5">
         <f>'[1]Dispatch details'!$L$2-'[1]Dispatch details'!$M$2</f>
         <v>1988590961.6160126</v>
       </c>
-      <c r="S4" s="5">
+      <c r="T4" s="5">
         <f>'[1]Dispatch details'!$N$2</f>
         <v>189570158.40000078</v>
       </c>
-      <c r="T4" s="5">
-        <f>R4-S4</f>
+      <c r="U4" s="5">
+        <f>S4-T4</f>
         <v>1799020803.2160118</v>
       </c>
-      <c r="U4" s="5">
+      <c r="V4" s="5">
         <v>1135435832.9599979</v>
       </c>
-      <c r="V4" s="5">
+      <c r="W4" s="5">
         <v>0</v>
       </c>
-      <c r="W4" s="5">
-        <f>U4-V4</f>
+      <c r="X4" s="5">
+        <f>V4-W4</f>
         <v>1135435832.9599979</v>
       </c>
     </row>
-    <row r="5" spans="2:23" x14ac:dyDescent="0.35">
+    <row r="5" spans="2:24" x14ac:dyDescent="0.35">
       <c r="B5" s="1" t="s">
         <v>10</v>
       </c>
@@ -2711,23 +2740,24 @@
       </c>
       <c r="P5" s="3"/>
       <c r="Q5" s="3"/>
-      <c r="R5" s="5">
+      <c r="R5" s="3"/>
+      <c r="S5" s="5">
         <f>'[2]Dispatch Tracker'!$O$2</f>
         <v>7243607.25</v>
       </c>
-      <c r="S5" s="5">
+      <c r="T5" s="5">
         <f>'[2]Payment details'!$C$3</f>
         <v>8000000</v>
       </c>
-      <c r="T5" s="5">
-        <f>R5-S5</f>
+      <c r="U5" s="5">
+        <f>S5-T5</f>
         <v>-756392.75</v>
       </c>
-      <c r="U5" s="5"/>
       <c r="V5" s="5"/>
       <c r="W5" s="5"/>
+      <c r="X5" s="5"/>
     </row>
-    <row r="6" spans="2:23" x14ac:dyDescent="0.35">
+    <row r="6" spans="2:24" x14ac:dyDescent="0.35">
       <c r="B6" s="1" t="s">
         <v>12</v>
       </c>
@@ -2772,17 +2802,18 @@
       </c>
       <c r="P6" s="3"/>
       <c r="Q6" s="3"/>
-      <c r="R6" s="5">
+      <c r="R6" s="3"/>
+      <c r="S6" s="5">
         <f>'[3]Dispatch Tracker'!$M$2-'[3]Dispatch Tracker'!$N$2</f>
         <v>411248281.60000002</v>
       </c>
-      <c r="S6" s="5"/>
       <c r="T6" s="5"/>
       <c r="U6" s="5"/>
       <c r="V6" s="5"/>
       <c r="W6" s="5"/>
+      <c r="X6" s="5"/>
     </row>
-    <row r="7" spans="2:23" x14ac:dyDescent="0.35">
+    <row r="7" spans="2:24" x14ac:dyDescent="0.35">
       <c r="B7" s="1" t="s">
         <v>13</v>
       </c>
@@ -2827,17 +2858,18 @@
       </c>
       <c r="P7" s="3"/>
       <c r="Q7" s="3"/>
-      <c r="R7" s="5">
+      <c r="R7" s="3"/>
+      <c r="S7" s="5">
         <f>'[4]Dispatch Tracker'!$M$2-'[4]Dispatch Tracker'!$N$2</f>
         <v>20291856</v>
       </c>
-      <c r="S7" s="5"/>
       <c r="T7" s="5"/>
       <c r="U7" s="5"/>
       <c r="V7" s="5"/>
       <c r="W7" s="5"/>
+      <c r="X7" s="5"/>
     </row>
-    <row r="8" spans="2:23" x14ac:dyDescent="0.35">
+    <row r="8" spans="2:24" x14ac:dyDescent="0.35">
       <c r="B8" s="1" t="s">
         <v>14</v>
       </c>
@@ -2882,23 +2914,24 @@
       </c>
       <c r="P8" s="3"/>
       <c r="Q8" s="3"/>
-      <c r="R8" s="5">
+      <c r="R8" s="3"/>
+      <c r="S8" s="5">
         <f>'[5]Dispatch tracker'!$T$3</f>
         <v>966549679.07200062</v>
       </c>
-      <c r="S8" s="5">
+      <c r="T8" s="5">
         <f>'[5]Dispatch tracker'!$Y$3</f>
         <v>883400238</v>
       </c>
-      <c r="T8" s="5">
-        <f>R8-S8</f>
+      <c r="U8" s="5">
+        <f>S8-T8</f>
         <v>83149441.072000623</v>
       </c>
-      <c r="U8" s="5"/>
       <c r="V8" s="5"/>
       <c r="W8" s="5"/>
+      <c r="X8" s="5"/>
     </row>
-    <row r="9" spans="2:23" x14ac:dyDescent="0.35">
+    <row r="9" spans="2:24" x14ac:dyDescent="0.35">
       <c r="B9" s="1" t="s">
         <v>16</v>
       </c>
@@ -2943,17 +2976,18 @@
       </c>
       <c r="P9" s="3"/>
       <c r="Q9" s="3"/>
-      <c r="R9" s="5">
+      <c r="R9" s="3"/>
+      <c r="S9" s="5">
         <f>'[6]Dispatch Tracker'!$O$2</f>
         <v>143794507.30000001</v>
       </c>
-      <c r="S9" s="5"/>
       <c r="T9" s="5"/>
       <c r="U9" s="5"/>
       <c r="V9" s="5"/>
       <c r="W9" s="5"/>
+      <c r="X9" s="5"/>
     </row>
-    <row r="10" spans="2:23" x14ac:dyDescent="0.35">
+    <row r="10" spans="2:24" x14ac:dyDescent="0.35">
       <c r="B10" s="1" t="s">
         <v>31</v>
       </c>
@@ -2970,7 +3004,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="11" spans="2:23" x14ac:dyDescent="0.35">
+    <row r="11" spans="2:24" x14ac:dyDescent="0.35">
       <c r="B11" s="1" t="s">
         <v>33</v>
       </c>
@@ -2987,7 +3021,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="12" spans="2:23" x14ac:dyDescent="0.35">
+    <row r="12" spans="2:24" x14ac:dyDescent="0.35">
       <c r="B12" s="1" t="s">
         <v>34</v>
       </c>

</xml_diff>